<commit_message>
chore: adoption report 2026-09-14 19:43 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-11</t>
+          <t>Quarter: Q3 2026  |  2026-09-14</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-15 18:41 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-14</t>
+          <t>Quarter: Q3 2026  |  2026-09-15</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-16 18:38 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-15</t>
+          <t>Quarter: Q3 2026  |  2026-09-16</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-17 18:45 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-16</t>
+          <t>Quarter: Q3 2026  |  2026-09-17</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-18 18:02 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-17</t>
+          <t>Quarter: Q3 2026  |  2026-09-18</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-21 19:51 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-18</t>
+          <t>Quarter: Q3 2026  |  2026-09-21</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-22 18:28 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-21</t>
+          <t>Quarter: Q3 2026  |  2026-09-22</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-23 18:48 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-22</t>
+          <t>Quarter: Q3 2026  |  2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-24 18:48 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-23</t>
+          <t>Quarter: Q3 2026  |  2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-25 19:06 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-24</t>
+          <t>Quarter: Q3 2026  |  2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-28 21:02 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-25</t>
+          <t>Quarter: Q3 2026  |  2026-09-28</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-29 00:46 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-28</t>
+          <t>Quarter: Q3 2026  |  2026-09-29</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-09-30 00:02 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-29</t>
+          <t>Quarter: Q3 2026  |  2026-09-30</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-01 00:18 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q3 2026  |  2026-09-30</t>
+          <t>Quarter: Q4 2026  |  2026-10-01</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2452,27 +2452,27 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Auto Efectivo</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>Ecommerce</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Ecommerce</t>
-        </is>
-      </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>64%</t>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -2481,24 +2481,24 @@
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>9789</v>
+        <v>0</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>15276</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Embebidos</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -2508,25 +2508,27 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>88%</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>34</v>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1424</v>
+        <v>9789</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>1625</v>
+        <v>15276</v>
       </c>
     </row>
     <row r="6">
@@ -2542,92 +2544,92 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q2 2026</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>34</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>0</v>
+        <v>1424</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="inlineStr">
-        <is>
-          <t>51%</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>22</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>3018</v>
+        <v>0</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>5891</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Embebidos</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2653,12 +2655,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -2673,31 +2675,31 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="F9" s="14" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>14419</v>
+        <v>3018</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>22099</v>
+        <v>5891</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Modelo Día</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2733,141 +2735,143 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Nueva Web Empresas</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Nueva Web Empresas</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>94%</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>17</v>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>172970</v>
+        <v>0</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>184326</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Nueva Web Empresas</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Nueva Web Empresas</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q2 2026</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>0</v>
+        <v>14419</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0</v>
+        <v>22099</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>84%</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>1</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>8539</v>
+        <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>10226</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Portal Digital de Siniestros</t>
+          <t>Modelo Día</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2893,12 +2897,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Protege 365</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Protege 365</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -2913,31 +2917,31 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="F15" s="14" t="n">
-        <v>317</v>
+        <v>17</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>7739</v>
+        <v>172970</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>8560</v>
+        <v>184326</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Protege 365</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Protege 365</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -2973,141 +2977,143 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Nueva Web Empresas</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>75%</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="n">
-        <v>615</v>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>1583</v>
+        <v>0</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>SOAT</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q2 2026</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>84%</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>0</v>
+        <v>8539</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0</v>
+        <v>10226</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Somos Corredores</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Somos Corredores</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="n">
-        <v>87</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>3852</v>
+        <v>0</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>4452</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Somos Corredores</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Somos Corredores</t>
+          <t>Portal Digital de Siniestros</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3133,12 +3139,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -3153,31 +3159,31 @@
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="F21" s="14" t="n">
-        <v>615</v>
+        <v>317</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>8</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>3906</v>
+        <v>7739</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>4593</v>
+        <v>8560</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>VDT</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -3213,46 +3219,48 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Protege 365</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>73%</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="n">
-        <v>615</v>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G23" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>2286</v>
+        <v>0</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>3132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Vehicular</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -3262,38 +3270,36 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q2 2026</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>615</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>0</v>
+        <v>1583</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>0</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -3303,36 +3309,38 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>69%</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="n">
-        <v>615</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G25" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>2650</v>
+        <v>0</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>3813</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Vehicular Todo Riesgo</t>
+          <t>SOAT</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -3342,12 +3350,12 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3373,12 +3381,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Venta Directa</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -3393,31 +3401,31 @@
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="F27" s="14" t="n">
-        <v>615</v>
+        <v>87</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>11370</v>
+        <v>3852</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>12076</v>
+        <v>4452</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Venta Directa</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -3453,46 +3461,48 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Ecommerce</t>
+          <t>Somos Corredores</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>85%</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="n">
-        <v>615</v>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>3566</v>
+        <v>0</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>4204</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Viajes</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -3502,111 +3512,716 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>Q2 2026</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>615</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>0</v>
+        <v>3906</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0</v>
+        <v>4593</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>VDT</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Web Corporativa</t>
+          <t>Ecommerce</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>84%</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="n">
-        <v>27</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>11472</v>
+        <v>0</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>13594</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>VDT</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>615</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>2286</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>3132</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>69%</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>615</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>2650</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>3813</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Vehicular Todo Riesgo</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Venta Directa</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>615</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>11370</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>12076</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Venta Directa</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Venta Directa</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>615</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>3566</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>4204</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Viajes</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Ecommerce</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
           <t>Web Corporativa</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>Web Corporativa</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>84%</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="H45" s="7" t="n">
+        <v>11472</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>13594</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Q3 2026</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="6" t="n">
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Web Corporativa</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: adoption report 2026-10-02 00:23 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-01</t>
+          <t>Quarter: Q4 2026  |  2026-10-02</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-03 00:05 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-02</t>
+          <t>Quarter: Q4 2026  |  2026-10-03</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-05 21:47 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-03</t>
+          <t>Quarter: Q4 2026  |  2026-10-05</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-06 01:37 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-05</t>
+          <t>Quarter: Q4 2026  |  2026-10-06</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-07 00:17 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-06</t>
+          <t>Quarter: Q4 2026  |  2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-08 00:39 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-07</t>
+          <t>Quarter: Q4 2026  |  2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-09 00:54 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-08</t>
+          <t>Quarter: Q4 2026  |  2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-10 00:25 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-09</t>
+          <t>Quarter: Q4 2026  |  2026-10-10</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-12 22:22 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-10</t>
+          <t>Quarter: Q4 2026  |  2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-13 02:20 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-12</t>
+          <t>Quarter: Q4 2026  |  2026-10-13</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-14 00:03 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-13</t>
+          <t>Quarter: Q4 2026  |  2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-15 18:51 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-14</t>
+          <t>Quarter: Q4 2026  |  2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-16 18:35 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-15</t>
+          <t>Quarter: Q4 2026  |  2026-10-16</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-19 20:20 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-16</t>
+          <t>Quarter: Q4 2026  |  2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-20 00:04 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-19</t>
+          <t>Quarter: Q4 2026  |  2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-21 19:05 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-20</t>
+          <t>Quarter: Q4 2026  |  2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-22 19:02 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-21</t>
+          <t>Quarter: Q4 2026  |  2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-23 18:51 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-22</t>
+          <t>Quarter: Q4 2026  |  2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-26 20:17 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-23</t>
+          <t>Quarter: Q4 2026  |  2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-27 00:09 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-26</t>
+          <t>Quarter: Q4 2026  |  2026-10-27</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-28 00:11 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-27</t>
+          <t>Quarter: Q4 2026  |  2026-10-28</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-29 00:33 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-28</t>
+          <t>Quarter: Q4 2026  |  2026-10-29</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-30 00:31 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-29</t>
+          <t>Quarter: Q4 2026  |  2026-10-30</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>

<commit_message>
chore: adoption report 2026-10-31 00:17 UTC
</commit_message>
<xml_diff>
--- a/docs/reporte-adopcion.xlsx
+++ b/docs/reporte-adopcion.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quarter: Q4 2026  |  2026-10-30</t>
+          <t>Quarter: Q4 2026  |  2026-10-31</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">

</xml_diff>